<commit_message>
feat: refactoring, test cases, enhancements
</commit_message>
<xml_diff>
--- a/deliverables/output/RIMSS - Estimation Sheet.xlsx
+++ b/deliverables/output/RIMSS - Estimation Sheet.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="134">
   <si>
     <t>Phase</t>
   </si>
@@ -251,6 +251,36 @@
     <t>Products, orders, push subscriptions; parameterized queries</t>
   </si>
   <si>
+    <t>Cart persistence, URL-synced search filters, debounced search, request cache</t>
+  </si>
+  <si>
+    <t>localStorage with validation; useSearchParams mirror; TTL cache with in-flight de-dup</t>
+  </si>
+  <si>
+    <t>Checkout flow: order placement from the cart drawer</t>
+  </si>
+  <si>
+    <t>orderService (non-retried POST), confirmation and error states</t>
+  </si>
+  <si>
+    <t>Accessibility hardening: focus-managed cart dialog, live regions, WCAG AA contrast</t>
+  </si>
+  <si>
+    <t>axe checks in Playwright</t>
+  </si>
+  <si>
+    <t>Telemetry beacon and global error capture; CSP/security headers</t>
+  </si>
+  <si>
+    <t>VITE_TELEMETRY_URL, public/_headers</t>
+  </si>
+  <si>
+    <t>Repo quality gates: Husky, lint-staged, commitlint, bundle budget, Dependabot, npm audit</t>
+  </si>
+  <si>
+    <t>Conventional Commits, pre-commit checks, CI budget</t>
+  </si>
+  <si>
     <t>Testing &amp; Bug Fixing Phase</t>
   </si>
   <si>
@@ -263,22 +293,22 @@
     <t>Component, service and module tests (Testing Library)</t>
   </si>
   <si>
-    <t>~77 tests covering loading/error/retry states</t>
+    <t>~110 tests covering loading/error/retry states, persistence, checkout and focus handling</t>
   </si>
   <si>
     <t>Backend API tests (supertest) incl. validation, security and pricing</t>
   </si>
   <si>
-    <t>~20 tests</t>
-  </si>
-  <si>
-    <t>Playwright end-to-end tests (desktop + mobile)</t>
+    <t>~40 tests</t>
+  </si>
+  <si>
+    <t>Playwright end-to-end tests (desktop + mobile, incl. axe accessibility)</t>
   </si>
   <si>
     <t>QA / Frontend Dev</t>
   </si>
   <si>
-    <t>~18 scenarios x 2 projects</t>
+    <t>~21 scenarios x 2 projects</t>
   </si>
   <si>
     <t>Push, offline and PWA install testing on real devices</t>
@@ -326,7 +356,7 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>≈ 64 person-days (13 person-weeks)</t>
+    <t>≈ 69 person-days (14 person-weeks)</t>
   </si>
   <si>
     <t>Category</t>
@@ -807,7 +837,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1379,10 +1409,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>30</v>
@@ -1391,267 +1421,352 @@
         <v>12</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D35" s="2">
+        <v>8</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D35" s="2">
-        <v>24</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D36" s="2">
+        <v>8</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D36" s="2">
-        <v>16</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D37" s="2">
+        <v>6</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D37" s="2">
-        <v>16</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="D38" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D39" s="2">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D40" s="2">
+        <v>24</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D40" s="2">
-        <v>16</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D41" s="2">
+        <v>16</v>
+      </c>
+      <c r="E41" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D41" s="2">
-        <v>8</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="D42" s="2">
         <v>16</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D43" s="2">
         <v>8</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>102</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D44" s="2">
+        <v>16</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D45" s="2">
+        <v>16</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>5</v>
+        <v>89</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>33</v>
+        <v>97</v>
       </c>
       <c r="D46" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>33</v>
+        <v>106</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>12</v>
+        <v>107</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>33</v>
+        <v>108</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>33</v>
+        <v>109</v>
       </c>
       <c r="D47" s="2">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>33</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>28</v>
+        <v>107</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>33</v>
+        <v>111</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>33</v>
+        <v>109</v>
       </c>
       <c r="D48" s="2">
-        <v>298</v>
+        <v>8</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D49" s="2">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D51" s="2">
+        <v>12</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D52" s="2">
+        <v>62</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D53" s="2">
+        <v>338</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D54" s="2">
         <v>116</v>
       </c>
-      <c r="E49" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D50" s="2">
+      <c r="E54" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D55" s="2">
         <v>24</v>
       </c>
-      <c r="E50" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D51" s="1">
-        <v>512</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>104</v>
+      <c r="E55" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D56" s="1">
+        <v>552</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1671,122 +1786,122 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: worked on tweaks
</commit_message>
<xml_diff>
--- a/deliverables/output/RIMSS - Estimation Sheet.xlsx
+++ b/deliverables/output/RIMSS - Estimation Sheet.xlsx
@@ -269,10 +269,10 @@
     <t>axe checks in Playwright</t>
   </si>
   <si>
-    <t>Telemetry beacon and global error capture; CSP/security headers</t>
-  </si>
-  <si>
-    <t>VITE_TELEMETRY_URL, public/_headers</t>
+    <t>Telemetry/analytics events stored locally via API JSON file; global error capture; log masking; CSP/security headers</t>
+  </si>
+  <si>
+    <t>VITE_TELEMETRY_URL (optional), public/_headers</t>
   </si>
   <si>
     <t>Repo quality gates: Husky, lint-staged, commitlint, bundle budget, Dependabot, npm audit</t>
@@ -413,7 +413,7 @@
     <t>Application is served over HTTPS (required for service workers and Web Push)</t>
   </si>
   <si>
-    <t>Telemetry backend (Sentry/App Insights) is provided by client; only the integration hook is estimated</t>
+    <t>Production telemetry/analytics collector (Sentry/App Insights) is provided by client; the sample stores events in a local JSON file via the API</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat: added few new features
</commit_message>
<xml_diff>
--- a/deliverables/output/RIMSS - Estimation Sheet.xlsx
+++ b/deliverables/output/RIMSS - Estimation Sheet.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="145">
   <si>
     <t>Phase</t>
   </si>
@@ -239,6 +239,39 @@
     <t>VAPID, admin-key protected broadcast</t>
   </si>
   <si>
+    <t>Backend: PostgreSQL persistence, migrations, idempotent orders, TLS options</t>
+  </si>
+  <si>
+    <t>Idempotency-Key header; JSON fallback without DATABASE_URL</t>
+  </si>
+  <si>
+    <t>Structured logging (pino) with masking, telemetry and analytics endpoint</t>
+  </si>
+  <si>
+    <t>NFR: observability</t>
+  </si>
+  <si>
+    <t>SCSS design tokens and shared ui/ components</t>
+  </si>
+  <si>
+    <t>Button, Card, Field, Heading, Table</t>
+  </si>
+  <si>
+    <t>Rule-based Chatbot assistant</t>
+  </si>
+  <si>
+    <t>responses.json intents; localStorage history</t>
+  </si>
+  <si>
+    <t>Dockerfiles and docker-compose (postgres, api, web)</t>
+  </si>
+  <si>
+    <t>DevOps</t>
+  </si>
+  <si>
+    <t>Multi-stage, non-root images</t>
+  </si>
+  <si>
     <t>Backend hardening: helmet, CORS allow-list, rate limiting, error envelope, config</t>
   </si>
   <si>
@@ -356,7 +389,7 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>≈ 69 person-days (14 person-weeks)</t>
+    <t>≈ 76 person-days (16 person-weeks)</t>
   </si>
   <si>
     <t>Category</t>
@@ -837,7 +870,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1384,7 +1417,7 @@
         <v>69</v>
       </c>
       <c r="D32" s="2">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>76</v>
@@ -1401,7 +1434,7 @@
         <v>69</v>
       </c>
       <c r="D33" s="2">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>78</v>
@@ -1449,13 +1482,13 @@
         <v>83</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="D36" s="2">
         <v>8</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1463,16 +1496,16 @@
         <v>28</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="D37" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1480,21 +1513,21 @@
         <v>28</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D38" s="2">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>90</v>
@@ -1511,7 +1544,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>92</v>
@@ -1520,7 +1553,7 @@
         <v>30</v>
       </c>
       <c r="D40" s="2">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>93</v>
@@ -1528,16 +1561,16 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="D41" s="2">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>95</v>
@@ -1545,84 +1578,84 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>96</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D42" s="2">
+        <v>6</v>
+      </c>
+      <c r="E42" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="D42" s="2">
-        <v>16</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D43" s="2">
+        <v>6</v>
+      </c>
+      <c r="E43" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D43" s="2">
-        <v>8</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D44" s="2">
+        <v>12</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D44" s="2">
-        <v>16</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>103</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D45" s="2">
+        <v>24</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="D45" s="2">
-        <v>16</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="D46" s="2">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>106</v>
@@ -1630,143 +1663,228 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="C47" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="D47" s="2">
         <v>16</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="D48" s="2">
         <v>8</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
         <v>112</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D49" s="2">
+        <v>16</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D50" s="2">
+        <v>16</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>33</v>
+        <v>108</v>
       </c>
       <c r="D51" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>33</v>
+        <v>117</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>12</v>
+        <v>118</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>33</v>
+        <v>119</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="D52" s="2">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>33</v>
+        <v>121</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>28</v>
+        <v>118</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>33</v>
+        <v>122</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="D53" s="2">
-        <v>338</v>
+        <v>8</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D54" s="2">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D56" s="2">
+        <v>12</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D57" s="2">
+        <v>62</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D58" s="2">
+        <v>390</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D59" s="2">
         <v>116</v>
       </c>
-      <c r="E54" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D55" s="2">
+      <c r="E59" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D60" s="2">
         <v>24</v>
       </c>
-      <c r="E55" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D56" s="1">
-        <v>552</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>114</v>
+      <c r="E60" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D61" s="1">
+        <v>604</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1786,122 +1904,122 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: added more enhancements
</commit_message>
<xml_diff>
--- a/deliverables/output/RIMSS - Estimation Sheet.xlsx
+++ b/deliverables/output/RIMSS - Estimation Sheet.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="222">
   <si>
     <t>Phase</t>
   </si>
@@ -314,6 +314,141 @@
     <t>Conventional Commits, pre-commit checks, CI budget</t>
   </si>
   <si>
+    <t>Authentication: register/login (scrypt, JWT), sign-in dialog, auth-gated checkout, account and order history</t>
+  </si>
+  <si>
+    <t>Frontend Dev / Backend Dev</t>
+  </si>
+  <si>
+    <t>Rate-limited auth routes, per-user order visibility, demo payment (pay/cancel)</t>
+  </si>
+  <si>
+    <t>Stock reservation: atomic decrement on order, restore on cancel, oversell protection</t>
+  </si>
+  <si>
+    <t>Conditional UPDATE in the order transaction; migration 003</t>
+  </si>
+  <si>
+    <t>Dark mode (CSS custom-property tokens) and English/Spanish i18n with persisted preferences</t>
+  </si>
+  <si>
+    <t>Theme toggle, language menu, message catalogue, contrast checks</t>
+  </si>
+  <si>
+    <t>Responsive header, active-nav highlighting, wishlist module, search paging</t>
+  </si>
+  <si>
+    <t>Stacked layout below desktop width</t>
+  </si>
+  <si>
+    <t>Technical documentation: ADRs, architecture views, README, generated deliverables</t>
+  </si>
+  <si>
+    <t>12 ADRs, Mermaid diagrams, Word/Excel deliverables</t>
+  </si>
+  <si>
+    <t>Infrastructure &amp; Environment Setup Phase</t>
+  </si>
+  <si>
+    <t>Infrastructure architecture, environment strategy and sizing (Dev, SIT, QA, UAT, Pre-prod, Prod, DR)</t>
+  </si>
+  <si>
+    <t>Architect / DevOps</t>
+  </si>
+  <si>
+    <t>Topology, promotion path, naming, capacity and cost plan</t>
+  </si>
+  <si>
+    <t>Infrastructure as code baseline: network, container registry, Kubernetes namespaces, shared modules</t>
+  </si>
+  <si>
+    <t>Reusable templates so every environment is built the same way</t>
+  </si>
+  <si>
+    <t>Dev environment: docker-compose, local Postgres, seed data, developer onboarding</t>
+  </si>
+  <si>
+    <t>DevOps / Frontend Dev</t>
+  </si>
+  <si>
+    <t>One-command start for web, API and database</t>
+  </si>
+  <si>
+    <t>SIT environment: web, API, managed Postgres, test data, integration endpoints</t>
+  </si>
+  <si>
+    <t>DevOps / QA</t>
+  </si>
+  <si>
+    <t>Shared integration environment, resettable data</t>
+  </si>
+  <si>
+    <t>QA environment: isolated deployment, data refresh and automation access</t>
+  </si>
+  <si>
+    <t>Hosts the Playwright and regression suites</t>
+  </si>
+  <si>
+    <t>UAT / Staging environment: production-like deployment with masked data</t>
+  </si>
+  <si>
+    <t>Business acceptance testing and release rehearsal</t>
+  </si>
+  <si>
+    <t>Pre-production / performance environment sized like production</t>
+  </si>
+  <si>
+    <t>Used for k6 load tests and failover checks</t>
+  </si>
+  <si>
+    <t>Production environment: hosting, autoscaling, CDN, WAF, managed Postgres with backups</t>
+  </si>
+  <si>
+    <t>Kubernetes manifests, ingress, HPA, high availability</t>
+  </si>
+  <si>
+    <t>Disaster recovery: backup and restore, multi-zone or secondary region, DR runbook and drill</t>
+  </si>
+  <si>
+    <t>RPO/RTO targets agreed with the client</t>
+  </si>
+  <si>
+    <t>DNS, TLS certificates and domain setup per environment</t>
+  </si>
+  <si>
+    <t>HTTPS is required for service workers and Web Push</t>
+  </si>
+  <si>
+    <t>Secrets and configuration management per environment (JWT_SECRET, VAPID keys, DATABASE_URL, CORS)</t>
+  </si>
+  <si>
+    <t>DevOps / Backend Dev</t>
+  </si>
+  <si>
+    <t>Secret store, rotation, no secrets in images or repo</t>
+  </si>
+  <si>
+    <t>Observability stack per environment: logs, metrics (/metrics), dashboards, alerts, telemetry collector</t>
+  </si>
+  <si>
+    <t>Prometheus-style metrics, structured log shipping, on-call alerts</t>
+  </si>
+  <si>
+    <t>Network and security hardening: firewall rules, least-privilege access, image scanning, access reviews</t>
+  </si>
+  <si>
+    <t>DevOps / Security</t>
+  </si>
+  <si>
+    <t>Trivy and CodeQL gates, private database access</t>
+  </si>
+  <si>
+    <t>Environment validation, smoke checks and handover documentation</t>
+  </si>
+  <si>
+    <t>Health checks, access matrix, environment runbooks</t>
+  </si>
+  <si>
     <t>Testing &amp; Bug Fixing Phase</t>
   </si>
   <si>
@@ -368,16 +503,97 @@
     <t>100ms interaction budget</t>
   </si>
   <si>
+    <t>Test strategy, test plan and test case design (functional, regression, NFR)</t>
+  </si>
+  <si>
+    <t>Traceability to requirements and NFRs</t>
+  </si>
+  <si>
+    <t>SIT execution: UI to API integration, checkout, auth, stock, push and offline flows</t>
+  </si>
+  <si>
+    <t>End-to-end scenarios across services, error and edge cases</t>
+  </si>
+  <si>
+    <t>SIT defect fixing and retest</t>
+  </si>
+  <si>
+    <t>Frontend Dev / Backend Dev / QA</t>
+  </si>
+  <si>
+    <t>Triage, fix, verify, regression</t>
+  </si>
+  <si>
+    <t>QA full regression cycle (desktop, tablet, mobile; Chrome, Edge, Firefox, Safari)</t>
+  </si>
+  <si>
+    <t>Includes dark mode and both languages</t>
+  </si>
+  <si>
+    <t>Security testing: OWASP Top 10 review, dependency audit, auth and rate-limit checks</t>
+  </si>
+  <si>
+    <t>QA / Backend Dev</t>
+  </si>
+  <si>
+    <t>npm audit, CodeQL, image scan, manual checks</t>
+  </si>
+  <si>
+    <t>Load and performance testing (k6) and tuning</t>
+  </si>
+  <si>
+    <t>Thresholds: p95 &lt; 300 ms, error rate &lt; 1%</t>
+  </si>
+  <si>
+    <t>Accessibility audit (WCAG 2.1 AA, keyboard and screen reader)</t>
+  </si>
+  <si>
+    <t>axe plus manual verification</t>
+  </si>
+  <si>
+    <t>UAT support, defect fixes and QA sign-off report</t>
+  </si>
+  <si>
+    <t>QA / TL</t>
+  </si>
+  <si>
+    <t>Business acceptance, exit criteria, test summary report</t>
+  </si>
+  <si>
+    <t>Release &amp; Deployment Phase</t>
+  </si>
+  <si>
+    <t>CD pipeline: image build, scan, deploy to staging and production</t>
+  </si>
+  <si>
+    <t>Trivy scan, environment promotion, rollback</t>
+  </si>
+  <si>
+    <t>Release readiness: release notes, runbook, rollback plan, go/no-go review</t>
+  </si>
+  <si>
+    <t>TL / PM</t>
+  </si>
+  <si>
+    <t>Production release and smoke test</t>
+  </si>
+  <si>
+    <t>Health, metrics and critical-path checks</t>
+  </si>
+  <si>
+    <t>Hypercare and post-release support</t>
+  </si>
+  <si>
+    <t>Monitoring, incident response, hotfixes during the first weeks</t>
+  </si>
+  <si>
     <t>Project Management</t>
   </si>
   <si>
     <t>Planning, status reporting, reviews</t>
   </si>
   <si>
-    <t>TL / PM</t>
-  </si>
-  <si>
-    <t>Across full 4-week duration</t>
+    <t>Across the full delivery, from planning through hypercare</t>
   </si>
   <si>
     <t>Risk management &amp; stakeholder communication</t>
@@ -389,7 +605,7 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>≈ 76 person-days (16 person-weeks)</t>
+    <t>≈ 138 person-days (28 person-weeks)</t>
   </si>
   <si>
     <t>Category</t>
@@ -413,6 +629,12 @@
     <t>Mock backend APIs for development/demo purposes</t>
   </si>
   <si>
+    <t>Test strategy, SIT, QA regression, security, load and accessibility testing, UAT support, release to staging/production and hypercare</t>
+  </si>
+  <si>
+    <t>Infrastructure setup for Dev, SIT, QA, UAT, Pre-prod, Production and DR: IaC, secrets, TLS/DNS, observability, backups and security hardening</t>
+  </si>
+  <si>
     <t>PWA (offline app shell), Web Push opt-in, resilient HTTP client, error boundaries, telemetry hook, feature flags, CI, Storybook</t>
   </si>
   <si>
@@ -422,7 +644,7 @@
     <t>Production push campaign tooling, audience segmentation and VAPID key management</t>
   </si>
   <si>
-    <t>Production hosting, managed Postgres provisioning/backups and payment processor (local docker-compose Postgres provided)</t>
+    <t>Payment processor integration and cloud cost/licence charges (infrastructure setup effort is in scope; the client supplies accounts and pays usage)</t>
   </si>
   <si>
     <t>Real payment processor integration and PCI compliance work</t>
@@ -441,6 +663,15 @@
   </si>
   <si>
     <t>Only evergreen browser support required (no IE11)</t>
+  </si>
+  <si>
+    <t>Cloud accounts, subscriptions, network access and domain ownership are provided by the client; infra effort assumes one cloud provider and Kubernetes</t>
+  </si>
+  <si>
+    <t>SIT and UAT environments, test users and business UAT participants are provided by the client</t>
+  </si>
+  <si>
+    <t>Hypercare is estimated for roughly the first two weeks after release; efforts are person-hours</t>
   </si>
   <si>
     <t>Application is served over HTTPS (required for service workers and Web Push)</t>
@@ -870,7 +1101,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1612,16 +1843,16 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="C44" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="D44" s="2">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>102</v>
@@ -1629,16 +1860,16 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>100</v>
+        <v>28</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>103</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="D45" s="2">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>104</v>
@@ -1646,16 +1877,16 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>100</v>
+        <v>28</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="D46" s="2">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>106</v>
@@ -1663,228 +1894,789 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>100</v>
+        <v>28</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>107</v>
       </c>
       <c r="C47" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D47" s="2">
+        <v>12</v>
+      </c>
+      <c r="E47" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="D47" s="2">
-        <v>16</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>100</v>
+        <v>28</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" s="2">
+        <v>16</v>
+      </c>
+      <c r="E48" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D48" s="2">
-        <v>8</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="D49" s="2">
         <v>16</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>115</v>
+        <v>84</v>
       </c>
       <c r="D50" s="2">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>33</v>
+        <v>116</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="D51" s="2">
         <v>8</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D52" s="2">
         <v>16</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D53" s="2">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D54" s="2">
+        <v>16</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D55" s="2">
+        <v>16</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>5</v>
+        <v>111</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>33</v>
+        <v>129</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="D56" s="2">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>33</v>
+        <v>130</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>12</v>
+        <v>111</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>33</v>
+        <v>131</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="D57" s="2">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>33</v>
+        <v>132</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>28</v>
+        <v>111</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>33</v>
+        <v>133</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="D58" s="2">
-        <v>390</v>
+        <v>8</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>33</v>
+        <v>134</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>33</v>
+        <v>135</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>33</v>
+        <v>136</v>
       </c>
       <c r="D59" s="2">
-        <v>116</v>
+        <v>12</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>33</v>
+        <v>137</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D60" s="2">
+        <v>20</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D61" s="2">
+        <v>16</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D62" s="2">
+        <v>8</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D63" s="2">
+        <v>12</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D64" s="2">
+        <v>24</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D65" s="2">
+        <v>16</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D66" s="2">
+        <v>16</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D67" s="2">
+        <v>8</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D68" s="2">
+        <v>16</v>
+      </c>
+      <c r="E68" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C60" s="2" t="s">
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D69" s="2">
+        <v>16</v>
+      </c>
+      <c r="E69" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D60" s="2">
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D70" s="2">
+        <v>8</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D71" s="2">
+        <v>16</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D72" s="2">
+        <v>32</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D73" s="2">
         <v>24</v>
       </c>
-      <c r="E60" s="2" t="s">
+      <c r="E73" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D74" s="2">
+        <v>24</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D75" s="2">
+        <v>16</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D76" s="2">
+        <v>12</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D77" s="2">
+        <v>8</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D78" s="2">
+        <v>16</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D79" s="2">
+        <v>12</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D80" s="2">
+        <v>8</v>
+      </c>
+      <c r="E80" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B61" s="5" t="s">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D81" s="2">
+        <v>8</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D82" s="2">
+        <v>24</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D83" s="2">
+        <v>16</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D84" s="2">
+        <v>8</v>
+      </c>
+      <c r="E84" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C61" s="5" t="s">
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B87" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D61" s="1">
-        <v>604</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>125</v>
+      <c r="C87" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D87" s="2">
+        <v>12</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D88" s="2">
+        <v>62</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D89" s="2">
+        <v>470</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D90" s="2">
+        <v>220</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D91" s="2">
+        <v>264</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D92" s="2">
+        <v>52</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D93" s="2">
+        <v>24</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B94" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C94" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D94" s="1">
+        <v>1104</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -1895,7 +2687,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1904,122 +2696,162 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>126</v>
+        <v>198</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>127</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>128</v>
+        <v>200</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>129</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>128</v>
+        <v>200</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>130</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>128</v>
+        <v>200</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>131</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>128</v>
+        <v>200</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>132</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>128</v>
+        <v>200</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>133</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>134</v>
+        <v>200</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>135</v>
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>134</v>
+        <v>200</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>136</v>
+        <v>207</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>137</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>138</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>139</v>
+        <v>208</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>140</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>139</v>
+        <v>208</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>141</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>139</v>
+        <v>213</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>142</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>139</v>
+        <v>213</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>143</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>139</v>
+        <v>213</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>144</v>
+        <v>216</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: worked on some enhancements
</commit_message>
<xml_diff>
--- a/deliverables/output/RIMSS - Estimation Sheet.xlsx
+++ b/deliverables/output/RIMSS - Estimation Sheet.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Estimation" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Assumptions &amp; Scope" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="AI Effort &amp; Tokens" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Assumptions &amp; Scope" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="237">
   <si>
     <t>Phase</t>
   </si>
@@ -302,10 +303,10 @@
     <t>axe checks in Playwright</t>
   </si>
   <si>
-    <t>Telemetry/analytics events stored locally via API JSON file; global error capture; log masking; CSP/security headers</t>
-  </si>
-  <si>
-    <t>VITE_TELEMETRY_URL (optional), public/_headers</t>
+    <t>Telemetry/analytics events stored locally via API JSON file and forwarded to Google Analytics 4 when configured; global error capture; log masking; CSP/security headers</t>
+  </si>
+  <si>
+    <t>VITE_TELEMETRY_URL (optional), VITE_GA_MEASUREMENT_ID (optional), public/_headers</t>
   </si>
   <si>
     <t>Repo quality gates: Husky, lint-staged, commitlint, bundle budget, Dependabot, npm audit</t>
@@ -341,6 +342,12 @@
     <t>Stacked layout below desktop width</t>
   </si>
   <si>
+    <t>Header product search with type-ahead suggestions and 30-minute inactivity sign-out</t>
+  </si>
+  <si>
+    <t>Debounced suggestions linking to product pages; activity-reset idle timer</t>
+  </si>
+  <si>
     <t>Technical documentation: ADRs, architecture views, README, generated deliverables</t>
   </si>
   <si>
@@ -605,7 +612,46 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>≈ 138 person-days (28 person-weeks)</t>
+    <t>≈ 139 person-days (28 person-weeks)</t>
+  </si>
+  <si>
+    <t>Manual Effort (Hours)</t>
+  </si>
+  <si>
+    <t>AI-assistable Share</t>
+  </si>
+  <si>
+    <t>AI-assisted Work (Hours)</t>
+  </si>
+  <si>
+    <t>Human Review (Hours)</t>
+  </si>
+  <si>
+    <t>Effort With AI (Hours)</t>
+  </si>
+  <si>
+    <t>Est. Input Tokens</t>
+  </si>
+  <si>
+    <t>Est. Output Tokens</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Saving: 495 hours (45%)</t>
+  </si>
+  <si>
+    <t>Token heuristic: 150,000 input and 20,000 output tokens per AI-assisted hour (agentic coding re-reads context on each step).</t>
+  </si>
+  <si>
+    <t>Human review adds 25% of each AI-assisted hour for review, testing and rework.</t>
+  </si>
+  <si>
+    <t>AI share per phase and token rates are planning assumptions, not measured usage; replace with actual usage from the AI tool dashboard.</t>
+  </si>
+  <si>
+    <t>Token cost depends on the model and pricing agreed with the client; costs are not included.</t>
   </si>
   <si>
     <t>Category</t>
@@ -684,6 +730,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -741,7 +790,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -756,6 +805,17 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1101,7 +1161,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1917,10 +1977,10 @@
         <v>109</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D48" s="2">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>110</v>
@@ -1928,33 +1988,33 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>112</v>
-      </c>
       <c r="C49" s="2" t="s">
-        <v>113</v>
+        <v>14</v>
       </c>
       <c r="D49" s="2">
         <v>16</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C50" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="D50" s="2">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>116</v>
@@ -1962,50 +2022,50 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>117</v>
       </c>
       <c r="C51" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D51" s="2">
+        <v>24</v>
+      </c>
+      <c r="E51" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="D51" s="2">
-        <v>8</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="D52" s="2">
+        <v>8</v>
+      </c>
+      <c r="E52" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="D52" s="2">
-        <v>16</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B53" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C53" s="2" t="s">
-        <v>121</v>
-      </c>
       <c r="D53" s="2">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>124</v>
@@ -2013,16 +2073,16 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>125</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>84</v>
+        <v>123</v>
       </c>
       <c r="D54" s="2">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>126</v>
@@ -2030,7 +2090,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>127</v>
@@ -2047,7 +2107,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>129</v>
@@ -2056,7 +2116,7 @@
         <v>84</v>
       </c>
       <c r="D56" s="2">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>130</v>
@@ -2064,7 +2124,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>131</v>
@@ -2073,7 +2133,7 @@
         <v>84</v>
       </c>
       <c r="D57" s="2">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>132</v>
@@ -2081,7 +2141,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>133</v>
@@ -2090,7 +2150,7 @@
         <v>84</v>
       </c>
       <c r="D58" s="2">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>134</v>
@@ -2098,33 +2158,33 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>135</v>
       </c>
       <c r="C59" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D59" s="2">
+        <v>8</v>
+      </c>
+      <c r="E59" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="D59" s="2">
-        <v>12</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="D60" s="2">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>139</v>
@@ -2132,33 +2192,33 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>140</v>
       </c>
       <c r="C61" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D61" s="2">
+        <v>20</v>
+      </c>
+      <c r="E61" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="D61" s="2">
-        <v>16</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="C62" s="2" t="s">
-        <v>121</v>
-      </c>
       <c r="D62" s="2">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>144</v>
@@ -2166,24 +2226,24 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="C63" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D63" s="2">
+        <v>8</v>
+      </c>
+      <c r="E63" s="2" t="s">
         <v>146</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D63" s="2">
-        <v>12</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>148</v>
@@ -2192,7 +2252,7 @@
         <v>30</v>
       </c>
       <c r="D64" s="2">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>149</v>
@@ -2200,16 +2260,16 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>150</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="D65" s="2">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>151</v>
@@ -2217,64 +2277,64 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>152</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>153</v>
+        <v>69</v>
       </c>
       <c r="D66" s="2">
         <v>16</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B67" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="D67" s="2">
+        <v>16</v>
+      </c>
+      <c r="E67" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="D67" s="2">
-        <v>8</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B68" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C68" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="C68" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="D68" s="2">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>33</v>
+        <v>159</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D69" s="2">
         <v>16</v>
@@ -2285,33 +2345,33 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>161</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="D70" s="2">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>162</v>
+        <v>33</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>163</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D71" s="2">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>164</v>
@@ -2319,16 +2379,16 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>165</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D72" s="2">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>166</v>
@@ -2336,30 +2396,30 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>167</v>
       </c>
       <c r="C73" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D73" s="2">
+        <v>32</v>
+      </c>
+      <c r="E73" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="D73" s="2">
-        <v>24</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B74" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="D74" s="2">
         <v>24</v>
@@ -2370,33 +2430,33 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C75" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D75" s="2">
+        <v>24</v>
+      </c>
+      <c r="E75" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="D75" s="2">
-        <v>16</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B76" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C76" s="2" t="s">
-        <v>173</v>
-      </c>
       <c r="D76" s="2">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>176</v>
@@ -2404,16 +2464,16 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>177</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="D77" s="2">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>178</v>
@@ -2421,84 +2481,84 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>179</v>
       </c>
       <c r="C78" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D78" s="2">
+        <v>8</v>
+      </c>
+      <c r="E78" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="D78" s="2">
-        <v>16</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="D79" s="2">
+        <v>16</v>
+      </c>
+      <c r="E79" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D79" s="2">
-        <v>12</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C80" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D80" s="2">
+        <v>12</v>
+      </c>
+      <c r="E80" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="D80" s="2">
-        <v>8</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>187</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>121</v>
+        <v>188</v>
       </c>
       <c r="D81" s="2">
         <v>8</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>188</v>
+        <v>33</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>189</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>168</v>
+        <v>123</v>
       </c>
       <c r="D82" s="2">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>190</v>
@@ -2506,63 +2566,63 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B83" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="C83" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D83" s="2">
+        <v>24</v>
+      </c>
+      <c r="E83" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D83" s="2">
-        <v>16</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D84" s="2">
+        <v>16</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D85" s="2">
         <v>8</v>
       </c>
-      <c r="E84" s="2" t="s">
+      <c r="E85" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" s="3" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D87" s="2">
-        <v>12</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>33</v>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" s="3" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>33</v>
@@ -2571,7 +2631,7 @@
         <v>33</v>
       </c>
       <c r="D88" s="2">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>33</v>
@@ -2579,7 +2639,7 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>33</v>
@@ -2588,7 +2648,7 @@
         <v>33</v>
       </c>
       <c r="D89" s="2">
-        <v>470</v>
+        <v>62</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>33</v>
@@ -2596,7 +2656,7 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>111</v>
+        <v>28</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>33</v>
@@ -2605,7 +2665,7 @@
         <v>33</v>
       </c>
       <c r="D90" s="2">
-        <v>220</v>
+        <v>478</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>33</v>
@@ -2613,7 +2673,7 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>145</v>
+        <v>113</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>33</v>
@@ -2622,7 +2682,7 @@
         <v>33</v>
       </c>
       <c r="D91" s="2">
-        <v>264</v>
+        <v>220</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>33</v>
@@ -2630,7 +2690,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>33</v>
@@ -2639,7 +2699,7 @@
         <v>33</v>
       </c>
       <c r="D92" s="2">
-        <v>52</v>
+        <v>264</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>33</v>
@@ -2647,7 +2707,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>33</v>
@@ -2656,27 +2716,44 @@
         <v>33</v>
       </c>
       <c r="D93" s="2">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="94" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="B94" s="5" t="s">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B94" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C94" s="5" t="s">
+      <c r="C94" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D94" s="1">
-        <v>1104</v>
-      </c>
-      <c r="E94" s="1" t="s">
-        <v>197</v>
+      <c r="D94" s="2">
+        <v>24</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C95" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D95" s="1">
+        <v>1112</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -2686,6 +2763,319 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="22" style="6" customWidth="1"/>
+    <col min="3" max="3" width="20" style="7" customWidth="1"/>
+    <col min="4" max="4" width="24" style="6" customWidth="1"/>
+    <col min="5" max="6" width="22" style="6" customWidth="1"/>
+    <col min="7" max="8" width="20" style="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="6">
+        <v>12</v>
+      </c>
+      <c r="C2" s="7">
+        <v>0.35</v>
+      </c>
+      <c r="D2" s="6">
+        <v>4.199999999999999</v>
+      </c>
+      <c r="E2" s="6">
+        <v>1.0499999999999998</v>
+      </c>
+      <c r="F2" s="6">
+        <v>8.850000000000001</v>
+      </c>
+      <c r="G2" s="8">
+        <v>630000</v>
+      </c>
+      <c r="H2" s="8">
+        <v>84000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="6">
+        <v>62</v>
+      </c>
+      <c r="C3" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="D3" s="6">
+        <v>24.8</v>
+      </c>
+      <c r="E3" s="6">
+        <v>6.2</v>
+      </c>
+      <c r="F3" s="6">
+        <v>43.400000000000006</v>
+      </c>
+      <c r="G3" s="8">
+        <v>3720000</v>
+      </c>
+      <c r="H3" s="8">
+        <v>496000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="6">
+        <v>478</v>
+      </c>
+      <c r="C4" s="7">
+        <v>0.7</v>
+      </c>
+      <c r="D4" s="6">
+        <v>334.59999999999997</v>
+      </c>
+      <c r="E4" s="6">
+        <v>83.64999999999999</v>
+      </c>
+      <c r="F4" s="6">
+        <v>227.05</v>
+      </c>
+      <c r="G4" s="8">
+        <v>50190000</v>
+      </c>
+      <c r="H4" s="8">
+        <v>6692000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="6">
+        <v>220</v>
+      </c>
+      <c r="C5" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="D5" s="6">
+        <v>110</v>
+      </c>
+      <c r="E5" s="6">
+        <v>27.5</v>
+      </c>
+      <c r="F5" s="6">
+        <v>137.5</v>
+      </c>
+      <c r="G5" s="8">
+        <v>16500000</v>
+      </c>
+      <c r="H5" s="8">
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" s="6">
+        <v>264</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="D6" s="6">
+        <v>158.4</v>
+      </c>
+      <c r="E6" s="6">
+        <v>39.6</v>
+      </c>
+      <c r="F6" s="6">
+        <v>145.2</v>
+      </c>
+      <c r="G6" s="8">
+        <v>23760000</v>
+      </c>
+      <c r="H6" s="8">
+        <v>3168000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" s="6">
+        <v>52</v>
+      </c>
+      <c r="C7" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="D7" s="6">
+        <v>20.8</v>
+      </c>
+      <c r="E7" s="6">
+        <v>5.2</v>
+      </c>
+      <c r="F7" s="6">
+        <v>36.4</v>
+      </c>
+      <c r="G7" s="8">
+        <v>3120000</v>
+      </c>
+      <c r="H7" s="8">
+        <v>416000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8" s="6">
+        <v>24</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="D8" s="6">
+        <v>7.199999999999999</v>
+      </c>
+      <c r="E8" s="6">
+        <v>1.7999999999999998</v>
+      </c>
+      <c r="F8" s="6">
+        <v>18.6</v>
+      </c>
+      <c r="G8" s="8">
+        <v>1080000</v>
+      </c>
+      <c r="H8" s="8">
+        <v>144000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B9" s="10">
+        <v>1112</v>
+      </c>
+      <c r="C9" s="11">
+        <v>0.5935251798561151</v>
+      </c>
+      <c r="D9" s="10">
+        <v>660</v>
+      </c>
+      <c r="E9" s="10">
+        <v>165</v>
+      </c>
+      <c r="F9" s="10">
+        <v>617</v>
+      </c>
+      <c r="G9" s="12">
+        <v>99000000</v>
+      </c>
+      <c r="H9" s="12">
+        <v>13200000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B11" s="14"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>209</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>210</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2695,163 +3085,163 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>199</v>
+      <c r="A1" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>201</v>
+      <c r="A2" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>202</v>
+      <c r="A3" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>203</v>
+      <c r="A4" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>204</v>
+      <c r="A5" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>205</v>
+      <c r="A6" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>206</v>
+      <c r="A7" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>207</v>
+      <c r="A8" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>209</v>
+      <c r="A9" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>210</v>
+      <c r="A10" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>211</v>
+      <c r="A11" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>212</v>
+      <c r="A12" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>214</v>
+      <c r="A13" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>215</v>
+      <c r="A14" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>216</v>
+      <c r="A15" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>217</v>
+      <c r="A16" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>218</v>
+      <c r="A17" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>219</v>
+      <c r="A18" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>220</v>
+      <c r="A19" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>221</v>
+      <c r="A20" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: worked on the UI and performance
</commit_message>
<xml_diff>
--- a/deliverables/output/RIMSS - Estimation Sheet.xlsx
+++ b/deliverables/output/RIMSS - Estimation Sheet.xlsx
@@ -174,7 +174,7 @@
     <t>NFR: fast repeat load, offline start-up</t>
   </si>
   <si>
-    <t>Web Push notifications (SW handlers, subscription client, header toggle, mock push endpoints)</t>
+    <t>Web Push notifications (SW handlers, subscription client, avatar-menu toggle, mock push endpoints)</t>
   </si>
   <si>
     <t>NFR: re-engagement; HTTPS + VAPID keys</t>
@@ -333,7 +333,7 @@
     <t>Dark mode (CSS custom-property tokens) and English/Spanish i18n with persisted preferences</t>
   </si>
   <si>
-    <t>Theme toggle, language menu, message catalogue, contrast checks</t>
+    <t>Theme toggle in avatar menu, language menu, message catalogue, contrast checks</t>
   </si>
   <si>
     <t>Responsive header, active-nav highlighting, wishlist module, search paging</t>

</xml_diff>